<commit_message>
Complete login module test cases
</commit_message>
<xml_diff>
--- a/Test_Cases/test_cases.xlsx
+++ b/Test_Cases/test_cases.xlsx
@@ -1,17 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Antoni\Desktop\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A3FC54F-98AD-469F-B2E8-E6F8A5E194C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-9700" yWindow="-21710" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Arkusz1" sheetId="1" r:id="rId5"/>
+    <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="65">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -52,23 +61,234 @@
     <t>TC-002</t>
   </si>
   <si>
-    <t>Login with invalid credentials</t>
+    <t>TC-003</t>
+  </si>
+  <si>
+    <t>TC-004</t>
+  </si>
+  <si>
+    <t>TC-005</t>
+  </si>
+  <si>
+    <t>TC-006</t>
+  </si>
+  <si>
+    <t>TC-007</t>
+  </si>
+  <si>
+    <t>TC-008</t>
+  </si>
+  <si>
+    <t>TC-009</t>
+  </si>
+  <si>
+    <t>TC-010</t>
+  </si>
+  <si>
+    <t>TC-011</t>
+  </si>
+  <si>
+    <t>TC-012</t>
+  </si>
+  <si>
+    <t>TC-013</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>User is on the login page</t>
+  </si>
+  <si>
+    <t>1. Enter username into the Username field.
+2. Enter password into the Password field.
+3. Click the Login button</t>
+  </si>
+  <si>
+    <t>Username: standard_user
+Password: secret_sauce</t>
+  </si>
+  <si>
+    <t>Username: standard_user
+Password: secret_sauce1</t>
+  </si>
+  <si>
+    <t>Login with valid username and invalid password</t>
+  </si>
+  <si>
+    <t>Login with valid password and empty Username field</t>
+  </si>
+  <si>
+    <t>Login with valid username and empty Password field</t>
+  </si>
+  <si>
+    <t>Login with empty Username and Password fields</t>
+  </si>
+  <si>
+    <t>Username: &lt;empty&gt;
+Password: secret_sauce</t>
+  </si>
+  <si>
+    <t>Username: standard_user
+Password: &lt;empty&gt;</t>
+  </si>
+  <si>
+    <t>Username: &lt;empty&gt;
+Password: &lt;empty&gt;</t>
+  </si>
+  <si>
+    <t>1. Enter username into the Username field.
+2. Leave the Password field empty.
+3. Click the Login button</t>
+  </si>
+  <si>
+    <t>1. Leave the Username fied empty.
+2. Enter password into the Password field.
+3. Click the Login button.</t>
+  </si>
+  <si>
+    <t>Login with valid password and invalid username</t>
+  </si>
+  <si>
+    <t>Username: standard_user1
+Password: secret_sauce</t>
+  </si>
+  <si>
+    <t>Login with locked out user</t>
+  </si>
+  <si>
+    <t>Login by pressing Enter</t>
+  </si>
+  <si>
+    <t>Login after multiple rapid clicks on Login button</t>
+  </si>
+  <si>
+    <t>Login with leading whitespace in Username</t>
+  </si>
+  <si>
+    <t>Login with leading whitespace in Password</t>
+  </si>
+  <si>
+    <t>Login with trailling whitespace in Password</t>
+  </si>
+  <si>
+    <t>Login with trailling whitespace in Username</t>
+  </si>
+  <si>
+    <t>`</t>
+  </si>
+  <si>
+    <t>1. Leave the Username field empty.
+2. Leave the Password field empty.
+3. Click the Login button</t>
+  </si>
+  <si>
+    <t>1. Enter username into the Username field.
+2. Enter password to the Password field.
+3. Click the Login button</t>
+  </si>
+  <si>
+    <t>Username: locked_out_user
+Password: secret_sauce</t>
+  </si>
+  <si>
+    <t>The user is redirected to the Inventory page. The inventory list is displayed, the "Products" page title is visible and the shopping cart icon are displayed.</t>
+  </si>
+  <si>
+    <t>The user remains on the Login page and is not redirected to the Inventory page. Instead, the following error message is displayed:"Epic sadface: Username and password do not match any user in this service".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The user remains on the Login page. Error message is displayed:"Epic sadface: Sorry, this user has been locked out.". User is not redirected to the Inventory page. </t>
+  </si>
+  <si>
+    <t>The user remains on the Login page. Error message is displayed: "Epic sadface: Username is required". User is not redirected to Inventory page. Validation indicators are displayed for required fields.</t>
+  </si>
+  <si>
+    <t>The user remains on the Login page. Error message is displayed: "Epic sadface: Password is required". User is not redirected to Inventory page. Validation indicators are displayed for required fields.</t>
+  </si>
+  <si>
+    <t>The user remains on the Login page. Error message is displayed: "Epic sadface: Username and password do not match any user in this service". User is not redirected to the Inventory page.</t>
+  </si>
+  <si>
+    <t>1. Enter username into the Username field.
+2. Enter password to the Password field.
+3. Press the Enter key.</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>1. Enter username into the Username field.
+2. Enter password to the Password field.
+3. Rapidly click the Login button 10 times.</t>
+  </si>
+  <si>
+    <t>The user is redirected to the Inventory page only once. The application remains responsive. User session is created only once. No error message displayed.</t>
+  </si>
+  <si>
+    <t>Username: &lt;leading space&gt;standard_user
+Password: secret_sauce</t>
+  </si>
+  <si>
+    <t>Username: standard_user&lt;trailling space&gt;
+Password: secret_sauce</t>
+  </si>
+  <si>
+    <t>Username: standard_user
+Password: &lt;leading space&gt;secret_sauce</t>
+  </si>
+  <si>
+    <t>Username: standard_user
+Password: secret_sauce&lt;trailling space&gt;</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -77,43 +297,129 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="7">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normalny" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="11">
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4FF0BA77-6979-4500-8BA1-C7F35D1F0E7A}" name="Tabela1" displayName="Tabela1" ref="A1:I14" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
+  <autoFilter ref="A1:I14" xr:uid="{4FF0BA77-6979-4500-8BA1-C7F35D1F0E7A}"/>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{88432B97-D4CF-451C-AD1C-ED6374D9F365}" name="Test Case ID" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{1D5378C8-4FEF-4098-A06C-0E643B6CD94E}" name="Module" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{F2C7497D-D66F-497C-A3C9-91150C1871C7}" name="Title" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{CB049A7F-17D9-4947-A00C-D05BEBE27E8E}" name="Preconditions" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{329AD1D2-9A6C-4B75-8731-35B632E67534}" name="Steps" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{8054514F-C4A7-46B9-AB42-BD141A431B00}" name="Test Data" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{47901A98-EDF9-4A26-864E-B36D51277682}" name="Expected Result" dataDxfId="2"/>
+    <tableColumn id="8" xr3:uid="{E75958DB-AB78-4E10-8CF6-7618D9899EF1}" name="Priority" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{8EA020A5-8A94-408D-A264-29FCA16CDFA5}" name="Status" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -303,71 +609,417 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:K14"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col customWidth="1" min="3" max="3" width="22.5"/>
+    <col min="1" max="1" width="12.6328125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="15.6328125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="35.6328125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="30.6328125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="50.6328125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="30.6328125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="40.6328125" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="12.6328125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:11" ht="50" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" s="2" t="s">
+      <c r="B2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="s">
+      <c r="D2" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I2" s="4"/>
+    </row>
+    <row r="3" spans="1:11" ht="62.5" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="2" t="s">
+      <c r="B3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I3" s="4"/>
+    </row>
+    <row r="4" spans="1:11" ht="62.5" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>13</v>
       </c>
+      <c r="B4" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I4" s="4"/>
+    </row>
+    <row r="5" spans="1:11" ht="62.5" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I5" s="4"/>
+      <c r="K5" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="62.5" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I6" s="4"/>
+    </row>
+    <row r="7" spans="1:11" ht="62.5" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I7" s="4"/>
+    </row>
+    <row r="8" spans="1:11" ht="50" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I8" s="4"/>
+    </row>
+    <row r="9" spans="1:11" ht="50" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="I9" s="4"/>
+    </row>
+    <row r="10" spans="1:11" ht="50" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="I10" s="4"/>
+    </row>
+    <row r="11" spans="1:11" ht="62.5" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I11" s="4"/>
+    </row>
+    <row r="12" spans="1:11" ht="62.5" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I12" s="4"/>
+    </row>
+    <row r="13" spans="1:11" ht="62.5" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I13" s="4"/>
+    </row>
+    <row r="14" spans="1:11" ht="62.5" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I14" s="4"/>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <phoneticPr fontId="4" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Expand manual test coverage for products cart and checkout
</commit_message>
<xml_diff>
--- a/Test_Cases/test_cases.xlsx
+++ b/Test_Cases/test_cases.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Antoni\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GitHub\manual-testing-ecommerce-app\Test_Cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A3FC54F-98AD-469F-B2E8-E6F8A5E194C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB78CC8F-7F90-413E-9DD7-594BD1DAF65E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-9700" yWindow="-21710" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="150">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -142,11 +142,6 @@
 3. Click the Login button</t>
   </si>
   <si>
-    <t>1. Leave the Username fied empty.
-2. Enter password into the Password field.
-3. Click the Login button.</t>
-  </si>
-  <si>
     <t>Login with valid password and invalid username</t>
   </si>
   <si>
@@ -240,6 +235,300 @@
   <si>
     <t>Username: standard_user
 Password: secret_sauce&lt;trailling space&gt;</t>
+  </si>
+  <si>
+    <t>TC-014</t>
+  </si>
+  <si>
+    <t>TC-015</t>
+  </si>
+  <si>
+    <t>TC-016</t>
+  </si>
+  <si>
+    <t>TC-017</t>
+  </si>
+  <si>
+    <t>TC-018</t>
+  </si>
+  <si>
+    <t>TC-019</t>
+  </si>
+  <si>
+    <t>TC-020</t>
+  </si>
+  <si>
+    <t>TC-021</t>
+  </si>
+  <si>
+    <t>TC-022</t>
+  </si>
+  <si>
+    <t>TC-023</t>
+  </si>
+  <si>
+    <t>TC-024</t>
+  </si>
+  <si>
+    <t>TC-025</t>
+  </si>
+  <si>
+    <t>Products</t>
+  </si>
+  <si>
+    <t>Products page opens correctly after successful login</t>
+  </si>
+  <si>
+    <t>User is on the login page.</t>
+  </si>
+  <si>
+    <t>1. Enter the username into the Username field.
+2. Enter the password into the Password field.
+3. Click the Login button.</t>
+  </si>
+  <si>
+    <t>User is successfully logged in and redirected to the Products page. The "Products" heading and product list are displayed.</t>
+  </si>
+  <si>
+    <t>Passed</t>
+  </si>
+  <si>
+    <t>All products are displayed correctly</t>
+  </si>
+  <si>
+    <t>User is logged in and is on the Products page.</t>
+  </si>
+  <si>
+    <t>1. Review the product list displayed on the Products page.
+2. Verify the image, name, description and price of each product.</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>All products are displayed. Each product has a corresponding image, name, description and price.</t>
+  </si>
+  <si>
+    <t>Product details page opens after clicking the product name</t>
+  </si>
+  <si>
+    <t>1. Click the "Sauce Labs Backpack" product name.</t>
+  </si>
+  <si>
+    <t>Product: Sauce Labs Backpack</t>
+  </si>
+  <si>
+    <t>The Product Details page for "Sauce Labs Backpack" is displayed. The product name, image, description and price are visible.</t>
+  </si>
+  <si>
+    <t>Product details page opens after clicking the product image</t>
+  </si>
+  <si>
+    <t>1. Click the "Sauce Labs Backpack" product image.</t>
+  </si>
+  <si>
+    <t>Sorting</t>
+  </si>
+  <si>
+    <t>Sorting by Name (A-Z) works correctly</t>
+  </si>
+  <si>
+    <t>1. Click the sorting dropdown.
+2. Select the "Name (A to Z)" option.</t>
+  </si>
+  <si>
+    <t>The products are sorted alphabetically by name in ascending order (A-Z).</t>
+  </si>
+  <si>
+    <t>Sorting by Price (Low to High) works correctly</t>
+  </si>
+  <si>
+    <t>1. Click the sorting dropdown.
+2. Select the "Price (low to high)" option.</t>
+  </si>
+  <si>
+    <t>The products are sorted by price in ascending order (low to high).</t>
+  </si>
+  <si>
+    <t>Cart</t>
+  </si>
+  <si>
+    <t>Adding a product to the cart works correctly</t>
+  </si>
+  <si>
+    <t>1. Click the "Add to cart" button for the "Sauce Labs Backpack" product.</t>
+  </si>
+  <si>
+    <t>The product is added to the cart. The cart counter increases by 1.</t>
+  </si>
+  <si>
+    <t>Removing a product from the cart works correctly</t>
+  </si>
+  <si>
+    <t>1. Click the "Add to cart" button for the "Sauce Labs Backpack" product.
+2. Click the cart icon.
+3. Click the "Remove" button for the "Sauce Labs Backpack" product.</t>
+  </si>
+  <si>
+    <t>The product is removed from the cart. The cart counter decreases by 1.</t>
+  </si>
+  <si>
+    <t>Cart counter updates correctly when multiple products are added and removed</t>
+  </si>
+  <si>
+    <t>1. Click the "Add to cart" button for the "Sauce Labs Backpack" product.
+2. Click the "Add to cart" button for the "Sauce Labs Bike Light" product.
+3. Verify the cart counter.
+4. Click the "Remove" button for the "Sauce Labs Backpack" product.
+5. Verify the cart counter.</t>
+  </si>
+  <si>
+    <t>Products: Sauce Labs Backpack, Sauce Labs Bike Light</t>
+  </si>
+  <si>
+    <t>The cart counter displays 1 after adding the first product and 2 after adding the second product. After removing one product, the cart counter decreases to 1.</t>
+  </si>
+  <si>
+    <t>Cart page opens after clicking the cart icon</t>
+  </si>
+  <si>
+    <t>1. Click the cart icon.</t>
+  </si>
+  <si>
+    <t>The Cart page is displayed with the "Your Cart" heading.</t>
+  </si>
+  <si>
+    <t>Checkout</t>
+  </si>
+  <si>
+    <t>Checkout page opens after clicking the Checkout button</t>
+  </si>
+  <si>
+    <t>User is logged in and is on the Cart page.</t>
+  </si>
+  <si>
+    <t>1. Click the Checkout button.</t>
+  </si>
+  <si>
+    <t>The Checkout: Your Information page is displayed with First Name, Last Name and Zip/Postal Code fields.</t>
+  </si>
+  <si>
+    <t>Continue checkout with valid customer informations</t>
+  </si>
+  <si>
+    <t>User is logged in, has at least one item in the cart and is on the Checkout: Your Information page.</t>
+  </si>
+  <si>
+    <t>First Name: Standard
+Last Name: User
+Zip/Postal Code: 1234</t>
+  </si>
+  <si>
+    <t>The user is redirected to the Checkout: Overview page.</t>
+  </si>
+  <si>
+    <t>TC-026</t>
+  </si>
+  <si>
+    <t>TC-027</t>
+  </si>
+  <si>
+    <t>TC-028</t>
+  </si>
+  <si>
+    <t>1. Leave the Username field empty.
+2. Enter password into the Password field.
+3. Click the Login button.</t>
+  </si>
+  <si>
+    <t>First Name: &lt;empty&gt;
+Last Name: User
+Zip/Postal Code: 1234</t>
+  </si>
+  <si>
+    <t>Continue checkout with empty First Name field</t>
+  </si>
+  <si>
+    <t>The user remains on the Checkout: Your Information page. The error message "Error: First Name is required" is displayed. The user is not redirected to the Checkout: Overview page. Validation indicators are displayed for required fields.</t>
+  </si>
+  <si>
+    <t>Continue checkout with empty Last Name field</t>
+  </si>
+  <si>
+    <t>The user remains on the Checkout: Your Information page. The error message "Error: Last Name is required" is displayed. The user is not redirected to the Checkout: Overview page. Validation indicators are displayed for required fields.</t>
+  </si>
+  <si>
+    <t>First Name: Standard
+Last Name: &lt;empty&gt;
+Zip/Postal Code: 1234</t>
+  </si>
+  <si>
+    <t>Continue checkout with empty Zip/Postal Code field</t>
+  </si>
+  <si>
+    <t>1. Enter the first name into the First Name field.
+2. Enter the last name into the Last Name field.
+3. Leave the Zip/Postal Code field empty.
+4. Click the "Continue" button.</t>
+  </si>
+  <si>
+    <t>First Name: Standard
+Last Name: User
+Zip/Postal Code: &lt;empty&gt;</t>
+  </si>
+  <si>
+    <t>The user remains on the Checkout: Your Information page. The error message "Error: Postal Code is required" is displayed. The user is not redirected to the Checkout: Overview page. Validation indicators are displayed for required fields.</t>
+  </si>
+  <si>
+    <t>1. Enter the first name into the First Name field.
+2. Enter the last name into the Last Name field.
+3. Enter the Zip/Postal Code into the Zip/Postal Code field.
+4. Click the "Continue" button.</t>
+  </si>
+  <si>
+    <t>1. Leave the First Name field empty.
+2. Enter the last name into the Last Name field.
+3. Enter the Zip/Postal Code into the Zip/Postal Code field.
+4. Click the "Continue" button.</t>
+  </si>
+  <si>
+    <t>1. Enter the first name into the First Name field.
+2. Leave the Last Name field empty.
+3. Enter the Zip/Postal Code into the Zip/Postal Code field.
+4. Click the "Continue" button.</t>
+  </si>
+  <si>
+    <t>TC-029</t>
+  </si>
+  <si>
+    <t>TC-030</t>
+  </si>
+  <si>
+    <t>Order completion</t>
+  </si>
+  <si>
+    <t>Checkout Overview displays correct order details</t>
+  </si>
+  <si>
+    <t>User is logged in, has at least one item in the cart and is on the Checkout: Overview page.</t>
+  </si>
+  <si>
+    <t>1. Review the products displayed in the order summary.
+2. Verify the item name, quantity and price.
+3. Verify the subtotal, tax and total values.</t>
+  </si>
+  <si>
+    <t>The Checkout: Overview page displays the correct product, quantity and price. The subtotal, tax and total values are displayed and calculated correctly.</t>
+  </si>
+  <si>
+    <t>Finalizing the order works correctly</t>
+  </si>
+  <si>
+    <t>1. Click the "Finish" button.
+2. Review the confirmation page.</t>
+  </si>
+  <si>
+    <t>The Checkout: Complete! page is displayed with a confirmation message. The "Back Home" and "Generate PDF order" buttons are displayed.</t>
   </si>
 </sst>
 </file>
@@ -401,8 +690,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4FF0BA77-6979-4500-8BA1-C7F35D1F0E7A}" name="Tabela1" displayName="Tabela1" ref="A1:I14" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
-  <autoFilter ref="A1:I14" xr:uid="{4FF0BA77-6979-4500-8BA1-C7F35D1F0E7A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4FF0BA77-6979-4500-8BA1-C7F35D1F0E7A}" name="Tabela1" displayName="Tabela1" ref="A1:I31" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
+  <autoFilter ref="A1:I31" xr:uid="{4FF0BA77-6979-4500-8BA1-C7F35D1F0E7A}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{88432B97-D4CF-451C-AD1C-ED6374D9F365}" name="Test Case ID" dataDxfId="8"/>
     <tableColumn id="2" xr3:uid="{1D5378C8-4FEF-4098-A06C-0E643B6CD94E}" name="Module" dataDxfId="7"/>
@@ -619,8 +908,8 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:K14"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:K31"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.6328125" style="1" customWidth="1"/>
     <col min="2" max="2" width="15.6328125" style="1" customWidth="1"/>
@@ -632,7 +921,7 @@
     <col min="8" max="16384" width="12.6328125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="13" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -681,12 +970,14 @@
         <v>27</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H2" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="I2" s="4"/>
+      <c r="I2" s="4" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="3" spans="1:11" ht="62.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
@@ -708,12 +999,14 @@
         <v>28</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H3" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="I3" s="4"/>
+      <c r="I3" s="4" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="4" spans="1:11" ht="62.5" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
@@ -723,7 +1016,7 @@
         <v>10</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>25</v>
@@ -732,15 +1025,17 @@
         <v>26</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H4" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="I4" s="4"/>
+      <c r="I4" s="4" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="5" spans="1:11" ht="62.5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
@@ -756,20 +1051,22 @@
         <v>25</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>37</v>
+        <v>126</v>
       </c>
       <c r="F5" s="6" t="s">
         <v>33</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H5" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="I5" s="4"/>
+      <c r="I5" s="4" t="s">
+        <v>81</v>
+      </c>
       <c r="K5" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="62.5" x14ac:dyDescent="0.25">
@@ -792,12 +1089,14 @@
         <v>34</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H6" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="I6" s="4"/>
+      <c r="I6" s="4" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="7" spans="1:11" ht="62.5" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
@@ -813,18 +1112,20 @@
         <v>25</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F7" s="6" t="s">
         <v>35</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H7" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="I7" s="4"/>
+      <c r="I7" s="4" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="8" spans="1:11" ht="50" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
@@ -834,24 +1135,26 @@
         <v>10</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>25</v>
       </c>
       <c r="E8" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F8" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="F8" s="4" t="s">
-        <v>50</v>
-      </c>
       <c r="G8" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H8" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="I8" s="4"/>
+      <c r="I8" s="4" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="9" spans="1:11" ht="50" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
@@ -861,24 +1164,26 @@
         <v>10</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>25</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F9" s="6" t="s">
         <v>27</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="I9" s="4"/>
+        <v>57</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="10" spans="1:11" ht="50" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
@@ -888,24 +1193,26 @@
         <v>10</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D10" s="4" t="s">
         <v>25</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>27</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="I10" s="4"/>
+        <v>57</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="11" spans="1:11" ht="62.5" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
@@ -915,7 +1222,7 @@
         <v>10</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>25</v>
@@ -924,15 +1231,17 @@
         <v>26</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H11" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="I11" s="4"/>
+      <c r="I11" s="4" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="12" spans="1:11" ht="62.5" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
@@ -942,7 +1251,7 @@
         <v>10</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>25</v>
@@ -951,15 +1260,17 @@
         <v>26</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H12" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="I12" s="4"/>
+      <c r="I12" s="4" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="13" spans="1:11" ht="62.5" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
@@ -969,7 +1280,7 @@
         <v>10</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D13" s="4" t="s">
         <v>25</v>
@@ -978,15 +1289,17 @@
         <v>26</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H13" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="I13" s="4"/>
+      <c r="I13" s="4" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="14" spans="1:11" ht="62.5" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
@@ -996,7 +1309,7 @@
         <v>10</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>25</v>
@@ -1005,15 +1318,510 @@
         <v>26</v>
       </c>
       <c r="F14" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="G14" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="H14" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="I14" s="4"/>
+      <c r="B15" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I15" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I16" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I17" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I18" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="25" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="I19" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="25" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="H20" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="I20" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="25" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="62.5" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="H22" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I22" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="100" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="H23" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I23" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="25" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="H24" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I24" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="H25" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I25" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="50" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="H26" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I26" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I27" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="G28" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="H28" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I28" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="G29" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="H29" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I29" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="50" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="G30" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="H30" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I30" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="G31" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="H31" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I31" s="4" t="s">
+        <v>81</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>

</xml_diff>